<commit_message>
Update MASTER Tournament Sheet.xlsx
</commit_message>
<xml_diff>
--- a/MASTER Tournament Sheet.xlsx
+++ b/MASTER Tournament Sheet.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="94">
   <si>
     <t>Tournament Name</t>
   </si>
@@ -131,6 +131,9 @@
   </si>
   <si>
     <t>Penalty</t>
+  </si>
+  <si>
+    <t>Point Deduction</t>
   </si>
   <si>
     <t>WRC</t>
@@ -256,7 +259,7 @@
     <t>8000 point penalty</t>
   </si>
   <si>
-    <t>Incorrect report sheet</t>
+    <t>Incorrect report sheet (report for each player)</t>
   </si>
   <si>
     <t>2000 point penalty each</t>
@@ -278,6 +281,21 @@
   </si>
   <si>
     <t>Forefiting a hanchan</t>
+  </si>
+  <si>
+    <t>CUSTOM</t>
+  </si>
+  <si>
+    <t>Custom Chombo</t>
+  </si>
+  <si>
+    <t>Custom Dead Hand</t>
+  </si>
+  <si>
+    <t>WRC (Lower Penalties)</t>
+  </si>
+  <si>
+    <t>Dead Hand</t>
   </si>
   <si>
     <t>Player #</t>
@@ -1017,9 +1035,11 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="23.5"/>
-    <col customWidth="1" min="3" max="3" width="30.13"/>
-    <col customWidth="1" min="4" max="4" width="12.75"/>
+    <col customWidth="1" min="1" max="1" width="6.63"/>
+    <col customWidth="1" min="2" max="2" width="32.5"/>
+    <col customWidth="1" min="3" max="3" width="54.5"/>
+    <col customWidth="1" min="4" max="4" width="23.0"/>
+    <col customWidth="1" min="5" max="5" width="12.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1035,425 +1055,1096 @@
       <c r="D1" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>41</v>
+      <c r="E3" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E4" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>46</v>
+      <c r="E6" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>46</v>
+      <c r="E7" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>46</v>
+      <c r="E8" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>46</v>
+      <c r="E11" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E13" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E19" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="E22" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>70</v>
+      <c r="E24" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
+      </c>
+      <c r="E27" s="1">
+        <v>-8.0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
+      </c>
+      <c r="E28" s="1">
+        <v>-2.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
+      </c>
+      <c r="E29" s="1">
+        <v>-1.0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
+      </c>
+      <c r="E30" s="1">
+        <v>-30.0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1">
+        <v>-30.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="1">
+        <v>-30.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E41" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E42" s="1">
+        <v>-20.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E44" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" s="1">
+        <v>-20.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E46" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E48" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E49" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E50" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E51" s="1">
+        <v>-20.0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E52" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E53" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E54" s="1">
+        <v>-20.0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E55" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E56" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E57" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E58" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E59" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E60" s="1">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E61" s="1">
+        <v>-1.0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>84</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E62" s="1">
+        <v>-30.0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E63" s="1">
+        <v>-30.0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E64" s="1">
+        <v>-20.0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E65" s="1">
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>
@@ -1470,10 +2161,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2">

</xml_diff>